<commit_message>
Corrigir Diretoria e auditoria do sistema.
Remove parentese extra na pagina Diretoria, corrige imports ao rodar inicializar_excel, testes das novas abas e verificacao de sintaxe no CI.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/apostolado.xlsx
+++ b/data/apostolado.xlsx
@@ -16,6 +16,12 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agenda" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Config" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Memorial" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Diretoria" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Zeladores" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Intencoes_Papa" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Centros" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comunicacoes" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reunioes" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -438,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N57"/>
+  <dimension ref="A1:R57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -455,6 +461,10 @@
     <col width="18" customWidth="1" min="12" max="12"/>
     <col width="18" customWidth="1" min="13" max="13"/>
     <col width="18" customWidth="1" min="14" max="14"/>
+    <col width="18" customWidth="1" min="15" max="15"/>
+    <col width="18" customWidth="1" min="16" max="16"/>
+    <col width="18" customWidth="1" min="17" max="17"/>
+    <col width="18" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -528,6 +538,26 @@
           <t>pagina</t>
         </is>
       </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>tipo_membro</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>comunidade</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>data_inscricao</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>fita_consagracao</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -585,6 +615,21 @@
       <c r="N2" t="inlineStr">
         <is>
           <t>p.6</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>Associado</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>Nova Odessa</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>Não</t>
         </is>
       </c>
     </row>
@@ -634,6 +679,17 @@
           <t>p.6</t>
         </is>
       </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>Associado</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr"/>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -689,6 +745,21 @@
           <t>p.6</t>
         </is>
       </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>Associado</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>Nova Odessa</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -749,6 +820,24 @@
       <c r="N5" t="inlineStr">
         <is>
           <t>p.6</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>Associado</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>Terranova</t>
+        </is>
+      </c>
+      <c r="Q5" s="2" t="n">
+        <v>42923</v>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>Não</t>
         </is>
       </c>
     </row>
@@ -798,6 +887,17 @@
           <t>p.6</t>
         </is>
       </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>Associado</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr"/>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -858,6 +958,24 @@
       <c r="N7" t="inlineStr">
         <is>
           <t>p.6</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>Associado</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>Jd. Fibra</t>
+        </is>
+      </c>
+      <c r="Q7" s="2" t="n">
+        <v>41640</v>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>Não</t>
         </is>
       </c>
     </row>
@@ -907,6 +1025,17 @@
           <t>p.6</t>
         </is>
       </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>Associado</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr"/>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -969,6 +1098,24 @@
           <t>p.6b</t>
         </is>
       </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>Associado</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>N. Sra. de Fátima</t>
+        </is>
+      </c>
+      <c r="Q9" s="2" t="n">
+        <v>42923</v>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -1031,6 +1178,24 @@
           <t>p.6b</t>
         </is>
       </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>Associado</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>N. Sra. de Fátima</t>
+        </is>
+      </c>
+      <c r="Q10" s="2" t="n">
+        <v>42923</v>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -1094,6 +1259,21 @@
           <t>p.6b</t>
         </is>
       </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>Associado</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>Santa Luíza II</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -1157,6 +1337,21 @@
           <t>p.6b</t>
         </is>
       </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>Associado</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>Nova Odessa</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -1212,6 +1407,21 @@
           <t>p.6b</t>
         </is>
       </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>Associado</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>N. Sra. de Fátima</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -1278,6 +1488,24 @@
           <t>p.6b</t>
         </is>
       </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>Associado</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>Santa Luíza II</t>
+        </is>
+      </c>
+      <c r="Q14" s="2" t="n">
+        <v>20090</v>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -1337,6 +1565,21 @@
           <t>p.7</t>
         </is>
       </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>Associado</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>Triunfo</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -1400,6 +1643,21 @@
           <t>p.7</t>
         </is>
       </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>Associado</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>Triunfo</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1459,6 +1717,21 @@
           <t>p.7</t>
         </is>
       </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>Associado</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>N. Sra. de Fátima</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1515,6 +1788,21 @@
           <t>p.7</t>
         </is>
       </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>Associado</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>N. Sra. de Fátima</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1574,6 +1862,21 @@
           <t>p.7</t>
         </is>
       </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>Associado</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>N. Sra. de Fátima</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1637,6 +1940,21 @@
           <t>p.7</t>
         </is>
       </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>Associado</t>
+        </is>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>Triunfo</t>
+        </is>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1692,6 +2010,21 @@
           <t>p.7b</t>
         </is>
       </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>Associado</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>Santa Luíza II</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1747,6 +2080,21 @@
           <t>p.7b</t>
         </is>
       </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>Associado</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>Santa Luíza II</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1802,6 +2150,21 @@
           <t>p.7b</t>
         </is>
       </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>Associado</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>Triunfo</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1865,6 +2228,21 @@
           <t>p.7b</t>
         </is>
       </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>Associado</t>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>Triunfo</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1915,6 +2293,21 @@
       <c r="N25" t="inlineStr">
         <is>
           <t>p.7b</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>Associado</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>Triunfo</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>Não</t>
         </is>
       </c>
     </row>
@@ -1964,6 +2357,17 @@
           <t>p.7b</t>
         </is>
       </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>Associado</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr"/>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -2015,6 +2419,17 @@
           <t>p.8</t>
         </is>
       </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>Associado</t>
+        </is>
+      </c>
+      <c r="P27" t="inlineStr"/>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -2064,6 +2479,17 @@
       <c r="N28" t="inlineStr">
         <is>
           <t>p.8</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>Associado</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr"/>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>Não</t>
         </is>
       </c>
     </row>
@@ -2113,6 +2539,17 @@
           <t>p.8</t>
         </is>
       </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>Associado</t>
+        </is>
+      </c>
+      <c r="P29" t="inlineStr"/>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -2157,6 +2594,17 @@
           <t>p.8</t>
         </is>
       </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>Associado</t>
+        </is>
+      </c>
+      <c r="P30" t="inlineStr"/>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -2204,6 +2652,17 @@
           <t>p.8</t>
         </is>
       </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>Associado</t>
+        </is>
+      </c>
+      <c r="P31" t="inlineStr"/>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -2248,6 +2707,17 @@
           <t>p.8</t>
         </is>
       </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>Associado</t>
+        </is>
+      </c>
+      <c r="P32" t="inlineStr"/>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -2292,6 +2762,17 @@
           <t>p.8b</t>
         </is>
       </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>Associado</t>
+        </is>
+      </c>
+      <c r="P33" t="inlineStr"/>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -2348,6 +2829,24 @@
       <c r="N34" t="inlineStr">
         <is>
           <t>p.8b</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>Associado</t>
+        </is>
+      </c>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>Santa Luíza I</t>
+        </is>
+      </c>
+      <c r="Q34" s="2" t="n">
+        <v>26665</v>
+      </c>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>Não</t>
         </is>
       </c>
     </row>
@@ -2397,6 +2896,17 @@
           <t>p.8b</t>
         </is>
       </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>Associado</t>
+        </is>
+      </c>
+      <c r="P35" t="inlineStr"/>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -2454,6 +2964,21 @@
       <c r="N36" t="inlineStr">
         <is>
           <t>p.8b</t>
+        </is>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>Associado</t>
+        </is>
+      </c>
+      <c r="P36" t="inlineStr">
+        <is>
+          <t>Triunfo</t>
+        </is>
+      </c>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>Não</t>
         </is>
       </c>
     </row>
@@ -2507,6 +3032,17 @@
           <t>p.8b</t>
         </is>
       </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>Associado</t>
+        </is>
+      </c>
+      <c r="P37" t="inlineStr"/>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -2560,6 +3096,21 @@
       <c r="N38" t="inlineStr">
         <is>
           <t>p.8b</t>
+        </is>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>Associado</t>
+        </is>
+      </c>
+      <c r="P38" t="inlineStr">
+        <is>
+          <t>N. Sra. de Fátima</t>
+        </is>
+      </c>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>Não</t>
         </is>
       </c>
     </row>
@@ -2609,6 +3160,17 @@
           <t>p.8b/9</t>
         </is>
       </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>Associado</t>
+        </is>
+      </c>
+      <c r="P39" t="inlineStr"/>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -2666,6 +3228,21 @@
       <c r="N40" t="inlineStr">
         <is>
           <t>p.9</t>
+        </is>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>Associado</t>
+        </is>
+      </c>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t>Terranova</t>
+        </is>
+      </c>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>Não</t>
         </is>
       </c>
     </row>
@@ -2715,6 +3292,17 @@
           <t>p.9</t>
         </is>
       </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>Associado</t>
+        </is>
+      </c>
+      <c r="P41" t="inlineStr"/>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -2774,6 +3362,21 @@
           <t>p.9</t>
         </is>
       </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>Associado</t>
+        </is>
+      </c>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>Triunfo</t>
+        </is>
+      </c>
+      <c r="R42" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -2833,6 +3436,21 @@
           <t>p.9</t>
         </is>
       </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>Associado</t>
+        </is>
+      </c>
+      <c r="P43" t="inlineStr">
+        <is>
+          <t>Triunfo</t>
+        </is>
+      </c>
+      <c r="R43" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -2890,6 +3508,21 @@
       <c r="N44" t="inlineStr">
         <is>
           <t>p.9</t>
+        </is>
+      </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>Associado</t>
+        </is>
+      </c>
+      <c r="P44" t="inlineStr">
+        <is>
+          <t>Santa Luíza I</t>
+        </is>
+      </c>
+      <c r="R44" t="inlineStr">
+        <is>
+          <t>Não</t>
         </is>
       </c>
     </row>
@@ -2939,6 +3572,17 @@
           <t>p.9</t>
         </is>
       </c>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>Associado</t>
+        </is>
+      </c>
+      <c r="P45" t="inlineStr"/>
+      <c r="R45" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -2996,6 +3640,21 @@
       <c r="N46" t="inlineStr">
         <is>
           <t>p.9b</t>
+        </is>
+      </c>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>Associado</t>
+        </is>
+      </c>
+      <c r="P46" t="inlineStr">
+        <is>
+          <t>Triunfo</t>
+        </is>
+      </c>
+      <c r="R46" t="inlineStr">
+        <is>
+          <t>Não</t>
         </is>
       </c>
     </row>
@@ -3045,6 +3704,17 @@
           <t>p.9b</t>
         </is>
       </c>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>Associado</t>
+        </is>
+      </c>
+      <c r="P47" t="inlineStr"/>
+      <c r="R47" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -3103,6 +3773,24 @@
           <t>p.9b</t>
         </is>
       </c>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>Associado</t>
+        </is>
+      </c>
+      <c r="P48" t="inlineStr">
+        <is>
+          <t>Santa Luíza II</t>
+        </is>
+      </c>
+      <c r="Q48" s="2" t="n">
+        <v>43525</v>
+      </c>
+      <c r="R48" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -3169,6 +3857,24 @@
           <t>p.9b</t>
         </is>
       </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>Associado</t>
+        </is>
+      </c>
+      <c r="P49" t="inlineStr">
+        <is>
+          <t>Jd. Fibra</t>
+        </is>
+      </c>
+      <c r="Q49" s="2" t="n">
+        <v>45814</v>
+      </c>
+      <c r="R49" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -3229,6 +3935,21 @@
           <t>p.9b</t>
         </is>
       </c>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>Associado</t>
+        </is>
+      </c>
+      <c r="P50" t="inlineStr">
+        <is>
+          <t>Triunfo</t>
+        </is>
+      </c>
+      <c r="R50" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -3291,6 +4012,24 @@
           <t>p.9b</t>
         </is>
       </c>
+      <c r="O51" t="inlineStr">
+        <is>
+          <t>Associado</t>
+        </is>
+      </c>
+      <c r="P51" t="inlineStr">
+        <is>
+          <t>Res. Fibra</t>
+        </is>
+      </c>
+      <c r="Q51" s="2" t="n">
+        <v>45814</v>
+      </c>
+      <c r="R51" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -3353,6 +4092,24 @@
           <t>p.10</t>
         </is>
       </c>
+      <c r="O52" t="inlineStr">
+        <is>
+          <t>Associado</t>
+        </is>
+      </c>
+      <c r="P52" t="inlineStr">
+        <is>
+          <t>Residencial Santa Luíza II</t>
+        </is>
+      </c>
+      <c r="Q52" s="2" t="n">
+        <v>46162</v>
+      </c>
+      <c r="R52" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -3419,6 +4176,24 @@
           <t>p.10</t>
         </is>
       </c>
+      <c r="O53" t="inlineStr">
+        <is>
+          <t>Associado</t>
+        </is>
+      </c>
+      <c r="P53" t="inlineStr">
+        <is>
+          <t>Terranova</t>
+        </is>
+      </c>
+      <c r="Q53" s="2" t="n">
+        <v>46060</v>
+      </c>
+      <c r="R53" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -3485,6 +4260,24 @@
           <t>p.10</t>
         </is>
       </c>
+      <c r="O54" t="inlineStr">
+        <is>
+          <t>Associado</t>
+        </is>
+      </c>
+      <c r="P54" t="inlineStr">
+        <is>
+          <t>Terranova</t>
+        </is>
+      </c>
+      <c r="Q54" s="2" t="n">
+        <v>46060</v>
+      </c>
+      <c r="R54" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -3551,6 +4344,24 @@
           <t>p.10</t>
         </is>
       </c>
+      <c r="O55" t="inlineStr">
+        <is>
+          <t>Associado</t>
+        </is>
+      </c>
+      <c r="P55" t="inlineStr">
+        <is>
+          <t>Santa Luíza I</t>
+        </is>
+      </c>
+      <c r="Q55" s="2" t="n">
+        <v>46166</v>
+      </c>
+      <c r="R55" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -3617,6 +4428,24 @@
           <t>p.10</t>
         </is>
       </c>
+      <c r="O56" t="inlineStr">
+        <is>
+          <t>Associado</t>
+        </is>
+      </c>
+      <c r="P56" t="inlineStr">
+        <is>
+          <t>Santa Luíza I</t>
+        </is>
+      </c>
+      <c r="Q56" s="2" t="n">
+        <v>46164</v>
+      </c>
+      <c r="R56" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -3678,6 +4507,689 @@
       <c r="N57" t="inlineStr">
         <is>
           <t>ficha</t>
+        </is>
+      </c>
+      <c r="O57" t="inlineStr">
+        <is>
+          <t>Associado</t>
+        </is>
+      </c>
+      <c r="P57" t="inlineStr">
+        <is>
+          <t>Santa Luíza I</t>
+        </is>
+      </c>
+      <c r="R57" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>cargo</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>nome</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>telefone</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>mandato_inicio</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>ativo</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>observacoes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Presidente</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Luiz Antônio</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" s="2" t="n">
+        <v>45812</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Coordenador</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Coordenadora</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Luíza Regina</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" s="2" t="n">
+        <v>45812</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Coordenadora pastoral</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Secretário(a)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>A preencher</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Tesoureiro(a)</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>A preencher</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Diretor Espiritual</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Pe. (paróquia)</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr"/>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Pároco ou indicado</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>membro_id</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>membro_nome</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>comunidade</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>data_posse</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>ativo</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>observacoes</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>mes</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>ano</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>titulo</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>texto</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>divulgada</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>observacoes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Intenções de June/2026</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Pela paz no mundo, pelos doentes, pelas famílias da paróquia e pelo Papa.</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Atualizar com o bilhete mensal / Mensageiro do Coração de Jesus</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>nome</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>comunidade</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>local</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>responsavel</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>telefone</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>ativo</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>observacoes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Centro Paróquia São Jorge</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Matriz</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Paróquia São Jorge</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Luiz Antônio</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Centro principal</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Centro Santa Luzia</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Santa Luzia</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Comunidade Santa Luzia</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Centro Santa Dulce</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Santa Dulce dos Pobres</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Comunidade Santa Dulce</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Centro N. Sra. de Fátima</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>N. Sra. de Fátima</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Comunidade N. Sra. de Fátima</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>tipo</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>titulo</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>mensagem</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>publico</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>registrado_por</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>observacoes</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>tipo</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>titulo</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>presentes</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>deliberacoes</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>ata_num</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>observacoes</t>
         </is>
       </c>
     </row>
@@ -5553,7 +7065,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:J1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -5564,6 +7076,8 @@
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
     <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5603,6 +7117,16 @@
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>tipo_visita</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>nota_pastoral</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>observacoes</t>
         </is>
@@ -5745,7 +7269,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -5754,6 +7278,8 @@
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5769,20 +7295,30 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>categoria</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>intencao</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>solicitante</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>prioridade</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>observacoes</t>
         </is>

</xml_diff>

<commit_message>
Atualizar cadastro completo a partir das fotos do livro.
Corrige nomes, telefones, enderecos e datas dos 56 membros; fichas Leila, Maria Neusa e Vera; comunidades pastorais.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/apostolado.xlsx
+++ b/data/apostolado.xlsx
@@ -22,6 +22,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Centros" sheetId="13" state="visible" r:id="rId13"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comunicacoes" sheetId="14" state="visible" r:id="rId14"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reunioes" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sugestoes" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reunioes_IA" sheetId="17" state="visible" r:id="rId17"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -622,11 +624,7 @@
           <t>Associado</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>Nova Odessa</t>
-        </is>
-      </c>
+      <c r="P2" t="inlineStr"/>
       <c r="R2" t="inlineStr">
         <is>
           <t>Não</t>
@@ -750,11 +748,7 @@
           <t>Associado</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>Nova Odessa</t>
-        </is>
-      </c>
+      <c r="P4" t="inlineStr"/>
       <c r="R4" t="inlineStr">
         <is>
           <t>Não</t>
@@ -814,7 +808,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>Paróquia Sta. Luzia – Pe. Luiz Antônio.</t>
+          <t>Pertence ao Apostolado desde 07/07/2017 – Paróquia Sta. Luzia – Pe. Luiz Antônio.</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -829,7 +823,7 @@
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>Terranova</t>
+          <t>Santa Luzia</t>
         </is>
       </c>
       <c r="Q5" s="2" t="n">
@@ -910,7 +904,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Cacilda Batista Degan</t>
+          <t>Cacilda Batista Pegan</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -967,7 +961,7 @@
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>Jd. Fibra</t>
+          <t>Santa Luzia</t>
         </is>
       </c>
       <c r="Q7" s="2" t="n">
@@ -1048,7 +1042,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Graziela Ellen Santos</t>
+          <t>Cristina Ellem Santos</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1057,7 +1051,7 @@
         </is>
       </c>
       <c r="E9" s="2" t="n">
-        <v>29228</v>
+        <v>29411</v>
       </c>
       <c r="F9" s="2" t="n">
         <v>42923</v>
@@ -1074,7 +1068,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>(19) 98147-46??</t>
+          <t>(19) 98117-4110</t>
         </is>
       </c>
       <c r="J9" t="inlineStr"/>
@@ -1090,7 +1084,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>Paróquia Sta. Luzia – Pe. Luís Antônio.</t>
+          <t>Pertence ao Apostolado desde 07/07/2017 – Paróquia Sta. Luzia – Pe. Luís Antônio.</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1105,7 +1099,7 @@
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>N. Sra. de Fátima</t>
+          <t>Santa Luzia</t>
         </is>
       </c>
       <c r="Q9" s="2" t="n">
@@ -1128,7 +1122,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Lucas Gaveta Silva</t>
+          <t>Lucas Caixeta Silva</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1170,7 +1164,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>Paróquia de Santa Luzia.</t>
+          <t>Pertence ao Apostolado desde 07/07/2017 – Paróquia de Santa Luzia – Pe. Luís Antônio.</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1185,7 +1179,7 @@
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>N. Sra. de Fátima</t>
+          <t>Santa Luzia</t>
         </is>
       </c>
       <c r="Q10" s="2" t="n">
@@ -1208,7 +1202,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Claudionice Batista Fernandes (Sau)</t>
+          <t>Claudionice Batista Fernandes (Jau)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1217,7 +1211,7 @@
         </is>
       </c>
       <c r="E11" s="2" t="n">
-        <v>26397</v>
+        <v>26488</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -1231,7 +1225,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>(19) 99528-3553</t>
+          <t>(19) 99528-3882</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -1251,7 +1245,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>Apelido: Sau. Comunidade Santa Luzia.</t>
+          <t>Apelido: Jau. Catequista – Comunidade Santa Luzia.</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -1266,7 +1260,7 @@
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>Santa Luíza II</t>
+          <t>Santa Luzia</t>
         </is>
       </c>
       <c r="R11" t="inlineStr">
@@ -1286,7 +1280,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Gleide</t>
+          <t>Cleide</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1295,7 +1289,7 @@
         </is>
       </c>
       <c r="E12" s="2" t="n">
-        <v>19316</v>
+        <v>19314</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -1304,7 +1298,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Nova Odessa</t>
+          <t>Triunfo</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1329,7 +1323,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>Atuou na Ministra da Eucaristia até 2019; hoje na Liturgia.</t>
+          <t>Ministra da Eucaristia até 2019; hoje na Liturgia.</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -1342,11 +1336,7 @@
           <t>Associado</t>
         </is>
       </c>
-      <c r="P12" t="inlineStr">
-        <is>
-          <t>Nova Odessa</t>
-        </is>
-      </c>
+      <c r="P12" t="inlineStr"/>
       <c r="R12" t="inlineStr">
         <is>
           <t>Não</t>
@@ -1373,7 +1363,7 @@
         </is>
       </c>
       <c r="E13" s="2" t="n">
-        <v>17458</v>
+        <v>17455</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
@@ -1443,7 +1433,7 @@
         </is>
       </c>
       <c r="E14" s="2" t="n">
-        <v>13329</v>
+        <v>13390</v>
       </c>
       <c r="F14" s="2" t="n">
         <v>20090</v>
@@ -1480,7 +1470,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>MEMBRO MAIS ANTIGO. Ingresso 1955 em Piracicaba; Nova Odessa desde 2000.</t>
+          <t>Pertence ao Apostolado desde 1955 (Itapevi, Par. São Judas Tadeu); Nova Odessa desde 2000. Filha: Vera (19) 98188-2997. Pastoral dos Doentes – Ministra da Eucaristia.</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -1495,7 +1485,7 @@
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>Santa Luíza II</t>
+          <t>Paróquia São Jorge</t>
         </is>
       </c>
       <c r="Q14" s="2" t="n">
@@ -1518,7 +1508,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Ione Michelan da Silva</t>
+          <t>Idione Michelan da Silva</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1531,7 +1521,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Rua Sebastião da Cruz Mata, 25</t>
+          <t>Rua Sebastião da Cruz Prata, 25</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1541,7 +1531,7 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>(19) 99320-4021</t>
+          <t>(19) 99320-4034</t>
         </is>
       </c>
       <c r="J15" t="inlineStr"/>
@@ -1570,11 +1560,7 @@
           <t>Associado</t>
         </is>
       </c>
-      <c r="P15" t="inlineStr">
-        <is>
-          <t>Triunfo</t>
-        </is>
-      </c>
+      <c r="P15" t="inlineStr"/>
       <c r="R15" t="inlineStr">
         <is>
           <t>Não</t>
@@ -1592,7 +1578,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Fátima Aparecida Felix Carmossi</t>
+          <t>Fátima Aparecida Felix Carmelossi</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1615,7 +1601,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>(19) 99384-5059</t>
+          <t>(19) 99384-5859</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -1635,7 +1621,7 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>Comunidade Sta. Luzia / Irmã Joyce.</t>
+          <t>Ministra da Eucaristia – Comunidade Sta. Luzia e Irmã Dulce.</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
@@ -1650,7 +1636,7 @@
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>Triunfo</t>
+          <t>Santa Luzia</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
@@ -1683,7 +1669,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Rua das Crianças, 1161</t>
+          <t>Rua das Crianças, 1164</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1744,7 +1730,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Sair Rosante</t>
+          <t>Jair Rosante</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1754,7 +1740,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Rua Jordano Milani, 158</t>
+          <t>Rua Jordano Milani, 148</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1780,7 +1766,7 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>Irmão de Helena Rosante (#17). Aniversário não preenchido.</t>
+          <t>Irmão de Helena Rosante (#17). Aniversário não preenchido no livro.</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
@@ -1838,7 +1824,7 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>(19) 99898-9562</t>
+          <t>(19) 99888-9562</t>
         </is>
       </c>
       <c r="J19" t="inlineStr"/>
@@ -1854,7 +1840,7 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>Possível filho de Helena (#17) e Osmar Caetano (#38).</t>
+          <t>Filho de Helena (#17) e Osmar Caetano (#38).</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
@@ -1889,7 +1875,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Jeanete Batista da Silva</t>
+          <t>Janete (Jeanete Batista da Silva)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1912,7 +1898,7 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>(19) 98158-3742</t>
+          <t>(19) 98138-3742</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -1932,7 +1918,7 @@
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>Pastoral Catequese – Coordenadora; Pastoral do Terço.</t>
+          <t>Pastoral Catequese (Coordenadora); Terço.</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
@@ -1945,11 +1931,7 @@
           <t>Associado</t>
         </is>
       </c>
-      <c r="P20" t="inlineStr">
-        <is>
-          <t>Triunfo</t>
-        </is>
-      </c>
+      <c r="P20" t="inlineStr"/>
       <c r="R20" t="inlineStr">
         <is>
           <t>Não</t>
@@ -1967,7 +1949,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Karen</t>
+          <t>Karla</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1980,7 +1962,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Rua Maximiliano Dal Medico, s/n</t>
+          <t>Rua Maximiliano Dal Medico</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -2002,7 +1984,7 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>Sobrenome não registrado.</t>
+          <t>Sobrenome não registrado no livro.</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
@@ -2015,11 +1997,7 @@
           <t>Associado</t>
         </is>
       </c>
-      <c r="P21" t="inlineStr">
-        <is>
-          <t>Santa Luíza II</t>
-        </is>
-      </c>
+      <c r="P21" t="inlineStr"/>
       <c r="R21" t="inlineStr">
         <is>
           <t>Não</t>
@@ -2060,7 +2038,7 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>(19) 99214-6855</t>
+          <t>(19) 99274-6853</t>
         </is>
       </c>
       <c r="J22" t="inlineStr"/>
@@ -2085,11 +2063,7 @@
           <t>Associado</t>
         </is>
       </c>
-      <c r="P22" t="inlineStr">
-        <is>
-          <t>Santa Luíza II</t>
-        </is>
-      </c>
+      <c r="P22" t="inlineStr"/>
       <c r="R22" t="inlineStr">
         <is>
           <t>Não</t>
@@ -2155,11 +2129,7 @@
           <t>Associado</t>
         </is>
       </c>
-      <c r="P23" t="inlineStr">
-        <is>
-          <t>Triunfo</t>
-        </is>
-      </c>
+      <c r="P23" t="inlineStr"/>
       <c r="R23" t="inlineStr">
         <is>
           <t>Não</t>
@@ -2230,14 +2200,10 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>Associado</t>
-        </is>
-      </c>
-      <c r="P24" t="inlineStr">
-        <is>
-          <t>Triunfo</t>
-        </is>
-      </c>
+          <t>Zelador</t>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr"/>
       <c r="R24" t="inlineStr">
         <is>
           <t>Não</t>
@@ -2300,11 +2266,7 @@
           <t>Associado</t>
         </is>
       </c>
-      <c r="P25" t="inlineStr">
-        <is>
-          <t>Triunfo</t>
-        </is>
-      </c>
+      <c r="P25" t="inlineStr"/>
       <c r="R25" t="inlineStr">
         <is>
           <t>Não</t>
@@ -2331,7 +2293,7 @@
         </is>
       </c>
       <c r="E26" s="2" t="n">
-        <v>26834</v>
+        <v>12316</v>
       </c>
       <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr"/>
@@ -2349,7 +2311,7 @@
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>Faleceu – data não registrada.</t>
+          <t>Faleceu – data do óbito não registrada no livro.</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
@@ -2389,7 +2351,7 @@
         </is>
       </c>
       <c r="E27" s="2" t="n">
-        <v>22709</v>
+        <v>22729</v>
       </c>
       <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr"/>
@@ -2411,7 +2373,7 @@
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>Endereço e telefone não preenchidos.</t>
+          <t>Coordenadora do Apostolado (livro: Lúcia Regina, 24/03/1962).</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
@@ -2421,7 +2383,7 @@
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>Associado</t>
+          <t>Zelador</t>
         </is>
       </c>
       <c r="P27" t="inlineStr"/>
@@ -2451,13 +2413,13 @@
         </is>
       </c>
       <c r="E28" s="2" t="n">
-        <v>15578</v>
+        <v>15609</v>
       </c>
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr"/>
       <c r="I28" t="inlineStr">
         <is>
-          <t>(19) 3486-1575</t>
+          <t>(19) 3466-1575</t>
         </is>
       </c>
       <c r="J28" t="inlineStr"/>
@@ -2785,7 +2747,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Nair Leal Damas</t>
+          <t>Nair Leal Domingos</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -2797,16 +2759,16 @@
         <v>14437</v>
       </c>
       <c r="F34" s="2" t="n">
-        <v>26665</v>
+        <v>33970</v>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Rua Dirceu Joc Boscori, 26</t>
+          <t>Rua Irineu José Zordon, 75</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>Santa Luíza I</t>
+          <t>Santa Luíza II</t>
         </is>
       </c>
       <c r="I34" t="inlineStr"/>
@@ -2823,7 +2785,7 @@
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>Participa do Apostolado desde 1973.</t>
+          <t>Participa do Apostolado desde 1993.</t>
         </is>
       </c>
       <c r="N34" t="inlineStr">
@@ -2836,13 +2798,9 @@
           <t>Associado</t>
         </is>
       </c>
-      <c r="P34" t="inlineStr">
-        <is>
-          <t>Santa Luíza I</t>
-        </is>
-      </c>
+      <c r="P34" t="inlineStr"/>
       <c r="Q34" s="2" t="n">
-        <v>26665</v>
+        <v>33970</v>
       </c>
       <c r="R34" t="inlineStr">
         <is>
@@ -2861,7 +2819,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Neuza Rafa</t>
+          <t>Neuza Rosa</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -2888,7 +2846,7 @@
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>Sobrenome 'Rafa' pode ser abreviação.</t>
+          <t>Endereço não informado no livro (NT).</t>
         </is>
       </c>
       <c r="N35" t="inlineStr">
@@ -2919,7 +2877,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Natália</t>
+          <t>Natalina</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -2942,7 +2900,7 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>(19) 99296-37??</t>
+          <t>(19) 99296-3723</t>
         </is>
       </c>
       <c r="J36" t="inlineStr"/>
@@ -2956,11 +2914,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="M36" t="inlineStr">
-        <is>
-          <t>Sobrenome não registrado.</t>
-        </is>
-      </c>
+      <c r="M36" t="inlineStr"/>
       <c r="N36" t="inlineStr">
         <is>
           <t>p.8b</t>
@@ -2971,11 +2925,7 @@
           <t>Associado</t>
         </is>
       </c>
-      <c r="P36" t="inlineStr">
-        <is>
-          <t>Triunfo</t>
-        </is>
-      </c>
+      <c r="P36" t="inlineStr"/>
       <c r="R36" t="inlineStr">
         <is>
           <t>Não</t>
@@ -3037,7 +2987,11 @@
           <t>Associado</t>
         </is>
       </c>
-      <c r="P37" t="inlineStr"/>
+      <c r="P37" t="inlineStr">
+        <is>
+          <t>Santa Luzia</t>
+        </is>
+      </c>
       <c r="R37" t="inlineStr">
         <is>
           <t>Não</t>
@@ -3055,7 +3009,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Osmar Caetano</t>
+          <t>Osmar Caetano (marido da Helena)</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -3064,7 +3018,7 @@
         </is>
       </c>
       <c r="E38" s="2" t="n">
-        <v>22738</v>
+        <v>22648</v>
       </c>
       <c r="G38" t="inlineStr">
         <is>
@@ -3134,7 +3088,7 @@
         </is>
       </c>
       <c r="E39" s="2" t="n">
-        <v>36559</v>
+        <v>37655</v>
       </c>
       <c r="G39" t="inlineStr"/>
       <c r="H39" t="inlineStr"/>
@@ -3152,7 +3106,7 @@
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>Registro fragmentado entre páginas 8b e 9.</t>
+          <t>Aniversário 03/02/2003 (livro p.9). Demais campos em branco.</t>
         </is>
       </c>
       <c r="N39" t="inlineStr">
@@ -3206,7 +3160,7 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>(19) 99825-5018</t>
+          <t>(19) 99525-5013</t>
         </is>
       </c>
       <c r="J40" t="inlineStr"/>
@@ -3237,7 +3191,7 @@
       </c>
       <c r="P40" t="inlineStr">
         <is>
-          <t>Terranova</t>
+          <t>Santa Luzia</t>
         </is>
       </c>
       <c r="R40" t="inlineStr">
@@ -3266,7 +3220,7 @@
         </is>
       </c>
       <c r="E41" s="2" t="n">
-        <v>17644</v>
+        <v>17705</v>
       </c>
       <c r="G41" t="inlineStr"/>
       <c r="H41" t="inlineStr"/>
@@ -3338,7 +3292,7 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>(19) 99287-6936</t>
+          <t>(19) 99287-6954</t>
         </is>
       </c>
       <c r="J42" t="inlineStr"/>
@@ -3354,7 +3308,7 @@
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t>Provável parente de Eurípia Frizoni (#43).</t>
+          <t>Mesmo endereço de Eurípia Frizoni (#43).</t>
         </is>
       </c>
       <c r="N42" t="inlineStr">
@@ -3367,11 +3321,7 @@
           <t>Associado</t>
         </is>
       </c>
-      <c r="P42" t="inlineStr">
-        <is>
-          <t>Triunfo</t>
-        </is>
-      </c>
+      <c r="P42" t="inlineStr"/>
       <c r="R42" t="inlineStr">
         <is>
           <t>Não</t>
@@ -3441,11 +3391,7 @@
           <t>Associado</t>
         </is>
       </c>
-      <c r="P43" t="inlineStr">
-        <is>
-          <t>Triunfo</t>
-        </is>
-      </c>
+      <c r="P43" t="inlineStr"/>
       <c r="R43" t="inlineStr">
         <is>
           <t>Não</t>
@@ -3515,11 +3461,7 @@
           <t>Associado</t>
         </is>
       </c>
-      <c r="P44" t="inlineStr">
-        <is>
-          <t>Santa Luíza I</t>
-        </is>
-      </c>
+      <c r="P44" t="inlineStr"/>
       <c r="R44" t="inlineStr">
         <is>
           <t>Não</t>
@@ -3595,7 +3537,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Isabel Ferreira Lopes (Izabel)</t>
+          <t>Izabel Ferreira Lopes (Izabel)</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -3618,7 +3560,7 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>(19) 99806-9342</t>
+          <t>(19) 98176-9772</t>
         </is>
       </c>
       <c r="J46" t="inlineStr"/>
@@ -3632,11 +3574,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="M46" t="inlineStr">
-        <is>
-          <t>Também grafada 'Izabel'.</t>
-        </is>
-      </c>
+      <c r="M46" t="inlineStr"/>
       <c r="N46" t="inlineStr">
         <is>
           <t>p.9b</t>
@@ -3647,11 +3585,7 @@
           <t>Associado</t>
         </is>
       </c>
-      <c r="P46" t="inlineStr">
-        <is>
-          <t>Triunfo</t>
-        </is>
-      </c>
+      <c r="P46" t="inlineStr"/>
       <c r="R46" t="inlineStr">
         <is>
           <t>Não</t>
@@ -3669,7 +3603,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Joanda</t>
+          <t>Iolanda</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -3696,7 +3630,7 @@
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>Grafia incomum – confirmar com membro.</t>
+          <t>Telefone e endereço não registrados.</t>
         </is>
       </c>
       <c r="N47" t="inlineStr">
@@ -3780,7 +3714,7 @@
       </c>
       <c r="P48" t="inlineStr">
         <is>
-          <t>Santa Luíza II</t>
+          <t>Paróquia São Jorge</t>
         </is>
       </c>
       <c r="Q48" s="2" t="n">
@@ -3812,7 +3746,7 @@
         </is>
       </c>
       <c r="E49" s="2" t="n">
-        <v>21480</v>
+        <v>21482</v>
       </c>
       <c r="F49" s="2" t="n">
         <v>45814</v>
@@ -3829,7 +3763,7 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>(19) 99765-890?</t>
+          <t>(19) 99765-4390</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
@@ -3849,7 +3783,7 @@
       </c>
       <c r="M49" t="inlineStr">
         <is>
-          <t>Pastoral Litúrgica – Irmã Joyce.</t>
+          <t>Membro do Apostolado desde 06/06/2025. Pastoral Litúrgica – Irmã Dulce.</t>
         </is>
       </c>
       <c r="N49" t="inlineStr">
@@ -3864,7 +3798,7 @@
       </c>
       <c r="P49" t="inlineStr">
         <is>
-          <t>Jd. Fibra</t>
+          <t>Santa Luzia</t>
         </is>
       </c>
       <c r="Q49" s="2" t="n">
@@ -3942,7 +3876,7 @@
       </c>
       <c r="P50" t="inlineStr">
         <is>
-          <t>Triunfo</t>
+          <t>Santa Luzia</t>
         </is>
       </c>
       <c r="R50" t="inlineStr">
@@ -3962,7 +3896,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Dana Rocha Santos</t>
+          <t>Daiana Rocha Santos</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -3988,7 +3922,7 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>(19) 99409-830?</t>
+          <t>(19) 99404-8130</t>
         </is>
       </c>
       <c r="J51" t="inlineStr"/>
@@ -4017,11 +3951,7 @@
           <t>Associado</t>
         </is>
       </c>
-      <c r="P51" t="inlineStr">
-        <is>
-          <t>Res. Fibra</t>
-        </is>
-      </c>
+      <c r="P51" t="inlineStr"/>
       <c r="Q51" s="2" t="n">
         <v>45814</v>
       </c>
@@ -4097,11 +4027,7 @@
           <t>Associado</t>
         </is>
       </c>
-      <c r="P52" t="inlineStr">
-        <is>
-          <t>Residencial Santa Luíza II</t>
-        </is>
-      </c>
+      <c r="P52" t="inlineStr"/>
       <c r="Q52" s="2" t="n">
         <v>46162</v>
       </c>
@@ -4133,27 +4059,24 @@
       <c r="E53" s="2" t="n">
         <v>24144</v>
       </c>
-      <c r="F53" s="2" t="n">
-        <v>46060</v>
-      </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>Rua da Amizade, 19</t>
+          <t>Rua da Amizade, 101</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>Terranova</t>
+          <t>Terra Nova</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>(19) 99466-2608</t>
+          <t>(19) 99466-3688</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>Ministra da Eucaristia – Comunidade Santa Dulce dos Pobres</t>
+          <t>Ministra da Eucaristia</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
@@ -4168,12 +4091,12 @@
       </c>
       <c r="M53" t="inlineStr">
         <is>
-          <t>Membro do Apostolado desde 07/02/2026.</t>
+          <t>Comunidade Santa Dulce dos Pobres. Participa de outra atividade pastoral: Ministra da Eucaristia. Ficha paróquia São Jorge.</t>
         </is>
       </c>
       <c r="N53" t="inlineStr">
         <is>
-          <t>p.10</t>
+          <t>ficha</t>
         </is>
       </c>
       <c r="O53" t="inlineStr">
@@ -4183,11 +4106,8 @@
       </c>
       <c r="P53" t="inlineStr">
         <is>
-          <t>Terranova</t>
-        </is>
-      </c>
-      <c r="Q53" s="2" t="n">
-        <v>46060</v>
+          <t>Santa Dulce dos Pobres</t>
+        </is>
       </c>
       <c r="R53" t="inlineStr">
         <is>
@@ -4217,9 +4137,6 @@
       <c r="E54" s="2" t="n">
         <v>24273</v>
       </c>
-      <c r="F54" s="2" t="n">
-        <v>46060</v>
-      </c>
       <c r="G54" t="inlineStr">
         <is>
           <t>Rua da Alegria, 542</t>
@@ -4227,17 +4144,17 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>Terranova</t>
+          <t>Terra Nova</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>(19) 99408-5202</t>
+          <t>(19) 99408-5302</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>Leiga Voluntária – Comunidade Santa Dulce dos Pobres</t>
+          <t>Leiga voluntária</t>
         </is>
       </c>
       <c r="K54" t="inlineStr">
@@ -4252,12 +4169,12 @@
       </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t>DESISTENTE – confirmado pelo coordenador. Consagrada na entrada.</t>
+          <t>Comunidade Santa Dulce dos Pobres. DESISTENTE. Leiga voluntária.</t>
         </is>
       </c>
       <c r="N54" t="inlineStr">
         <is>
-          <t>p.10</t>
+          <t>ficha</t>
         </is>
       </c>
       <c r="O54" t="inlineStr">
@@ -4267,15 +4184,12 @@
       </c>
       <c r="P54" t="inlineStr">
         <is>
-          <t>Terranova</t>
-        </is>
-      </c>
-      <c r="Q54" s="2" t="n">
-        <v>46060</v>
+          <t>Santa Dulce dos Pobres</t>
+        </is>
       </c>
       <c r="R54" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
     </row>
@@ -4346,12 +4260,12 @@
       </c>
       <c r="O55" t="inlineStr">
         <is>
-          <t>Associado</t>
+          <t>Zelador</t>
         </is>
       </c>
       <c r="P55" t="inlineStr">
         <is>
-          <t>Santa Luíza I</t>
+          <t>Santa Luzia</t>
         </is>
       </c>
       <c r="Q55" s="2" t="n">
@@ -4359,7 +4273,7 @@
       </c>
       <c r="R55" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
     </row>
@@ -4374,7 +4288,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Vera Lucia de Abreu Lobão</t>
+          <t>Vera Lúcia de Abreu Rodão</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -4385,9 +4299,6 @@
       <c r="E56" s="2" t="n">
         <v>28310</v>
       </c>
-      <c r="F56" s="2" t="n">
-        <v>46164</v>
-      </c>
       <c r="G56" t="inlineStr">
         <is>
           <t>Rua Ângelo Piconi, 471</t>
@@ -4405,7 +4316,7 @@
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>Pastoral do Batismo – Paróquia São Jorge</t>
+          <t>Pastoral do Batismo</t>
         </is>
       </c>
       <c r="K56" t="inlineStr">
@@ -4420,12 +4331,12 @@
       </c>
       <c r="M56" t="inlineStr">
         <is>
-          <t>Consagrada em 05/06/2026. Verificar duplicidade com Irene Pedrao (C2).</t>
+          <t>Comunidade Santa Luiza. Pastoral do Batismo. Consagrada em 05/06/2026. Verificar duplicidade com Irene Pedrao (C2).</t>
         </is>
       </c>
       <c r="N56" t="inlineStr">
         <is>
-          <t>p.10</t>
+          <t>ficha</t>
         </is>
       </c>
       <c r="O56" t="inlineStr">
@@ -4435,15 +4346,12 @@
       </c>
       <c r="P56" t="inlineStr">
         <is>
-          <t>Santa Luíza I</t>
-        </is>
-      </c>
-      <c r="Q56" s="2" t="n">
-        <v>46164</v>
+          <t>Santa Luzia</t>
+        </is>
       </c>
       <c r="R56" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
     </row>
@@ -4514,11 +4422,7 @@
           <t>Associado</t>
         </is>
       </c>
-      <c r="P57" t="inlineStr">
-        <is>
-          <t>Santa Luíza I</t>
-        </is>
-      </c>
+      <c r="P57" t="inlineStr"/>
       <c r="R57" t="inlineStr">
         <is>
           <t>Não</t>
@@ -5198,6 +5102,156 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>autor</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>tipo</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>texto</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>resposta</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>observacoes</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>titulo</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>arquivo_audio</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>transcricao_arquivo</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>duracao_min</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>resumo</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>explicacao</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>pontos_chave</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>observacoes</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -5524,7 +5578,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Cacilda(#6), Graziela(#9), Natália(#36), Marlene(#49), Dana(#51) – dígitos ilegíveis.</t>
+          <t>Cacilda(#6) – último dígito ilegível no livro.</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -5622,7 +5676,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Grafia incomum</t>
+          <t>Grafia no livro</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -5632,17 +5686,17 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Joanda(#47); Neuza Rafa(#35).</t>
+          <t>Lúcia/Luíza Regina (#27); Izabel/Iolanda conforme livro físico.</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Confirmar grafia oficial.</t>
+          <t>Registro atualizado pelas fotos do livro.</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
     </row>
@@ -5659,7 +5713,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Luiz Antônio(#24) &amp; Iara(#25); família Rosante-Caetano; Frizoni; Graziela &amp; Lucas; Rosangela &amp; Carlos.</t>
+          <t>Luiz Antônio(#24) &amp; Iara(#25); família Rosante-Caetano; Frizoni; Cristina &amp; Lucas (#9–10); Rosangela &amp; Carlos.</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -5869,7 +5923,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Joanda</t>
+          <t>Iolanda</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -5944,7 +5998,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Neuza Rafa</t>
+          <t>Neuza Rosa</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -6019,7 +6073,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Cacilda Batista Degan</t>
+          <t>Cacilda Batista Pegan</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -6073,11 +6127,11 @@
         <v>13</v>
       </c>
       <c r="B14" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Devanira Vitta Lobão</t>
+          <t>Cristina Ellem Santos</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -6102,11 +6156,11 @@
         <v>14</v>
       </c>
       <c r="B15" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Graziela Ellen Santos</t>
+          <t>Devanira Vitta Lobão</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -6160,11 +6214,11 @@
         <v>16</v>
       </c>
       <c r="B17" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Jefferson Ap. Rosante Caetano</t>
+          <t>Jair Rosante</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -6189,11 +6243,11 @@
         <v>17</v>
       </c>
       <c r="B18" t="n">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Lucas Gaveta Silva</t>
+          <t>Jefferson Ap. Rosante Caetano</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -6218,11 +6272,11 @@
         <v>18</v>
       </c>
       <c r="B19" t="n">
-        <v>38</v>
+        <v>10</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Osmar Caetano</t>
+          <t>Lucas Caixeta Silva</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -6247,11 +6301,11 @@
         <v>19</v>
       </c>
       <c r="B20" t="n">
-        <v>18</v>
+        <v>38</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Sair Rosante</t>
+          <t>Osmar Caetano (marido da Helena)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -6305,11 +6359,11 @@
         <v>21</v>
       </c>
       <c r="B22" t="n">
-        <v>12</v>
+        <v>51</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Gleide</t>
+          <t>Daiana Rocha Santos</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -6325,7 +6379,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Nova Odessa</t>
+          <t>Res. Fibra</t>
         </is>
       </c>
     </row>
@@ -6334,11 +6388,11 @@
         <v>22</v>
       </c>
       <c r="B23" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Dana Rocha Santos</t>
+          <t>Carlos José Amorim Nobuyasu</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -6354,7 +6408,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Res. Fibra</t>
+          <t>Residencial Santa Luíza II</t>
         </is>
       </c>
     </row>
@@ -6363,11 +6417,11 @@
         <v>23</v>
       </c>
       <c r="B24" t="n">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Carlos José Amorim Nobuyasu</t>
+          <t>Eliane Francisca dos Santos</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -6383,7 +6437,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Residencial Santa Luíza II</t>
+          <t>Santa Luíza I</t>
         </is>
       </c>
     </row>
@@ -6392,11 +6446,11 @@
         <v>24</v>
       </c>
       <c r="B25" t="n">
-        <v>55</v>
+        <v>102</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Eliane Francisca dos Santos</t>
+          <t>Irene Rosineia de Abreu Pedrao</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -6421,11 +6475,11 @@
         <v>25</v>
       </c>
       <c r="B26" t="n">
-        <v>102</v>
+        <v>44</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Irene Rosineia de Abreu Pedrao</t>
+          <t>Valdomira Marestoni (D. Nena)</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -6450,11 +6504,11 @@
         <v>26</v>
       </c>
       <c r="B27" t="n">
-        <v>34</v>
+        <v>56</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Nair Leal Damas</t>
+          <t>Vera Lúcia de Abreu Rodão</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -6479,11 +6533,11 @@
         <v>27</v>
       </c>
       <c r="B28" t="n">
-        <v>44</v>
+        <v>11</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Valdomira Marestoni (D. Nena)</t>
+          <t>Claudionice Batista Fernandes (Jau)</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -6499,7 +6553,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Santa Luíza I</t>
+          <t>Santa Luíza II</t>
         </is>
       </c>
     </row>
@@ -6508,11 +6562,11 @@
         <v>28</v>
       </c>
       <c r="B29" t="n">
-        <v>56</v>
+        <v>14</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Vera Lucia de Abreu Lobão</t>
+          <t>Eneide Bernardes Grandini</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -6528,7 +6582,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Santa Luíza I</t>
+          <t>Santa Luíza II</t>
         </is>
       </c>
     </row>
@@ -6537,11 +6591,11 @@
         <v>29</v>
       </c>
       <c r="B30" t="n">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Claudionice Batista Fernandes (Sau)</t>
+          <t>Karla</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -6566,11 +6620,11 @@
         <v>30</v>
       </c>
       <c r="B31" t="n">
-        <v>14</v>
+        <v>34</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Eneide Bernardes Grandini</t>
+          <t>Nair Leal Domingos</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -6595,11 +6649,11 @@
         <v>31</v>
       </c>
       <c r="B32" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Karen</t>
+          <t>Renata Cristina Rodrigues Scardovelli</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -6624,11 +6678,11 @@
         <v>32</v>
       </c>
       <c r="B33" t="n">
-        <v>22</v>
+        <v>48</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Renata Cristina Rodrigues Scardovelli</t>
+          <t>Rosangela Alves Amorim de Oliveira</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -6653,11 +6707,11 @@
         <v>33</v>
       </c>
       <c r="B34" t="n">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Rosangela Alves Amorim de Oliveira</t>
+          <t>Leila Barbosa Fonseca</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -6673,7 +6727,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Santa Luíza II</t>
+          <t>Terra Nova</t>
         </is>
       </c>
     </row>
@@ -6711,11 +6765,11 @@
         <v>35</v>
       </c>
       <c r="B36" t="n">
-        <v>53</v>
+        <v>40</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Leila Barbosa Fonseca</t>
+          <t>Osinete Aparecida dos Santos</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -6740,11 +6794,11 @@
         <v>36</v>
       </c>
       <c r="B37" t="n">
-        <v>40</v>
+        <v>12</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Osinete Aparecida dos Santos</t>
+          <t>Cleide</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -6760,7 +6814,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Terranova</t>
+          <t>Triunfo</t>
         </is>
       </c>
     </row>
@@ -6802,7 +6856,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Fátima Aparecida Felix Carmossi</t>
+          <t>Fátima Aparecida Felix Carmelossi</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -6860,7 +6914,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Isabel Ferreira Lopes (Izabel)</t>
+          <t>Izabel Ferreira Lopes (Izabel)</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -6889,7 +6943,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Jeanete Batista da Silva</t>
+          <t>Janete (Jeanete Batista da Silva)</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -7005,7 +7059,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Natália</t>
+          <t>Natalina</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -7206,7 +7260,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>DESISTENTE – confirmado pelo coordenador. Consagrada na entrada.</t>
+          <t>Comunidade Santa Dulce dos Pobres. DESISTENTE. Leiga voluntária.</t>
         </is>
       </c>
     </row>
@@ -7243,7 +7297,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Vera Lucia de Abreu Lobão</t>
+          <t>Vera Lúcia de Abreu Rodão</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
@@ -7254,7 +7308,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Consagrada em 05/06/2026. Verificar duplicidade com Irene Pedrao (C2).</t>
+          <t>Comunidade Santa Luiza. Pastoral do Batismo. Consagrada em 05/06/2026. Verificar duplicidade com Irene Pedrao (C2).</t>
         </is>
       </c>
     </row>
@@ -7645,11 +7699,11 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>26834</v>
+        <v>12316</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>#26 – Faleceu – data não registrada</t>
+          <t>#26 – Faleceu – data do óbito não registrada</t>
         </is>
       </c>
     </row>

</xml_diff>